<commit_message>
Update ECY through August 2026
</commit_message>
<xml_diff>
--- a/ecy4.xlsx
+++ b/ecy4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://perissosprivatewealth-my.sharepoint.com/personal/brandon_perissosprivatewealth_com/Documents/1 Perissos Private Wealth Management/5 Python/01_Active_Strategies/Wealth Utility API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="418" documentId="13_ncr:1_{A317B0E7-1C5D-450E-A529-DF31A54AA737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E0B27F3-1BEB-4DCC-822C-B34D4988B4E8}"/>
+  <xr:revisionPtr revIDLastSave="585" documentId="13_ncr:1_{A317B0E7-1C5D-450E-A529-DF31A54AA737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A348269F-7370-4258-894B-78847219CA50}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="15840" windowWidth="28800" windowHeight="15840" activeTab="1" xr2:uid="{7D23DFD4-FCD3-40E1-B8A0-B864FE11F7D6}"/>
+    <workbookView xWindow="28695" yWindow="15840" windowWidth="29010" windowHeight="15945" activeTab="1" xr2:uid="{7D23DFD4-FCD3-40E1-B8A0-B864FE11F7D6}"/>
   </bookViews>
   <sheets>
     <sheet name="ecy" sheetId="2" r:id="rId1"/>
@@ -945,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{173E5D82-F300-41D6-89B7-1A964CE4FD56}">
-  <dimension ref="A1:F557"/>
+  <dimension ref="A1:F561"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -977,15 +977,15 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
-        <f t="array" ref="A2:A557">_xll.YCDS("I:SP500ECY",,"1980-01-01")</f>
+        <f t="array" ref="A2:A561">_xll.YCDS("I:SP500ECY",,"1980-01-01")</f>
         <v>1980-01-31</v>
       </c>
       <c r="B2">
-        <f t="array" aca="1" ref="B2:B557" ca="1">_xll.YCS("I:SP500ECY",,"1980-01-01")</f>
+        <f t="array" aca="1" ref="B2:B561" ca="1">_xll.YCS("I:SP500ECY",,"1980-01-01")</f>
         <v>7.9799999999999996E-2</v>
       </c>
       <c r="C2">
-        <f t="array" aca="1" ref="C2:C557" ca="1">_xll.YCS("I:usltir",,"1980-01-01")</f>
+        <f t="array" aca="1" ref="C2:C561" ca="1">_xll.YCS("I:usltir",,"1980-01-01")</f>
         <v>0.108</v>
       </c>
       <c r="D2">
@@ -993,7 +993,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="E2" s="1">
-        <f t="array" aca="1" ref="E2:E556" ca="1">_xll.YCS("I:us1mccpi",,"1980-01-01")</f>
+        <f t="array" aca="1" ref="E2:E560" ca="1">_xll.YCS("I:us1mccpi",,"1980-01-01")</f>
         <v>1.4E-2</v>
       </c>
       <c r="F2" s="1">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="B554">
         <f ca="1"/>
-        <v>1.54E-2</v>
+        <v>1.5299999999999999E-2</v>
       </c>
       <c r="C554">
         <f ca="1"/>
@@ -14771,7 +14771,7 @@
       </c>
       <c r="B555">
         <f ca="1"/>
-        <v>1.7000000000000001E-2</v>
+        <v>1.6899999999999998E-2</v>
       </c>
       <c r="C555">
         <f ca="1"/>
@@ -14788,7 +14788,7 @@
       </c>
       <c r="B556">
         <f ca="1"/>
-        <v>1.67E-2</v>
+        <v>1.77E-2</v>
       </c>
       <c r="C556">
         <f ca="1"/>
@@ -14805,11 +14805,79 @@
       </c>
       <c r="B557">
         <f ca="1"/>
-        <v>1.6400000000000001E-2</v>
+        <v>1.66E-2</v>
       </c>
       <c r="C557">
         <f ca="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.3200000000000002E-2</v>
+      </c>
+      <c r="E557" s="1">
+        <f ca="1"/>
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="558" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A558" t="str">
+        <v>2026-05-31</v>
+      </c>
+      <c r="B558">
+        <f ca="1"/>
+        <v>1.3899999999999999E-2</v>
+      </c>
+      <c r="C558">
+        <f ca="1"/>
+        <v>4.48E-2</v>
+      </c>
+      <c r="E558" s="1">
+        <f ca="1"/>
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="559" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A559" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="B559">
+        <f ca="1"/>
+        <v>1.3100000000000001E-2</v>
+      </c>
+      <c r="C559">
+        <f ca="1"/>
+        <v>4.4699999999999997E-2</v>
+      </c>
+      <c r="E559" s="1">
+        <f ca="1"/>
+        <v>-4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="560" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A560" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="B560">
+        <f ca="1"/>
+        <v>1.18E-2</v>
+      </c>
+      <c r="C560">
+        <f ca="1"/>
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="E560" s="1">
+        <f ca="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="561" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A561" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="B561">
+        <f ca="1"/>
+        <v>9.7000000000000003E-3</v>
+      </c>
+      <c r="C561">
+        <f ca="1"/>
+        <v>4.7500000000000001E-2</v>
       </c>
     </row>
   </sheetData>
@@ -14819,14 +14887,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA56A079-CA0B-477E-8FC4-5F43798C1EE5}">
-  <dimension ref="A1:J677"/>
+  <dimension ref="A1:J681"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14864,7 +14932,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
-        <f t="array" ref="A2:A677">_xll.YCDS("I:USLTIR",,"1970-01-31")</f>
+        <f t="array" ref="A2:A681">_xll.YCDS("I:USLTIR",,"1970-01-31")</f>
         <v>1970-01-31</v>
       </c>
       <c r="B2">
@@ -14872,11 +14940,11 @@
         <v>48.877504749340375</v>
       </c>
       <c r="C2">
-        <f t="array" aca="1" ref="C2:C676" ca="1">_xll.YCS("I:USCPI",,"1970-01-31")</f>
+        <f t="array" aca="1" ref="C2:C680" ca="1">_xll.YCS("I:USCPI",,"1970-01-31")</f>
         <v>37.9</v>
       </c>
       <c r="D2">
-        <f t="array" aca="1" ref="D2:D677" ca="1">_xll.YCS("I:USLTIR",,"1970-01-31")</f>
+        <f t="array" aca="1" ref="D2:D681" ca="1">_xll.YCS("I:USLTIR",,"1970-01-31")</f>
         <v>7.7899999999999997E-2</v>
       </c>
       <c r="E2">
@@ -14895,11 +14963,11 @@
         <v>1.0916666666666661E-3</v>
       </c>
       <c r="I2" s="2">
-        <f t="array" aca="1" ref="I2:I677" ca="1">_xll.YCS("I:SP500ECY",,"1970-01-31")</f>
+        <f t="array" aca="1" ref="I2:I681" ca="1">_xll.YCS("I:SP500ECY",,"1970-01-31")</f>
         <v>6.4000000000000003E-3</v>
       </c>
       <c r="J2" s="2">
-        <f t="array" aca="1" ref="J2:J676" ca="1">_xll.YCS("I:SP500RD", ,"1970-01-31")</f>
+        <f t="array" aca="1" ref="J2:J679" ca="1">_xll.YCS("I:SP500RD", ,"1970-01-31")</f>
         <v>21.813400000000001</v>
       </c>
     </row>
@@ -41107,7 +41175,7 @@
         <v>2023-05-31</v>
       </c>
       <c r="B642">
-        <f t="shared" ref="B642:B669" ca="1" si="40">F642*$C$669/C642</f>
+        <f t="shared" ref="B642:B680" ca="1" si="40">F642*$C$669/C642</f>
         <v>190.85561928493718</v>
       </c>
       <c r="C642">
@@ -41160,7 +41228,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
       <c r="E643">
-        <f t="shared" ref="E643:E669" ca="1" si="41">D643/12</f>
+        <f t="shared" ref="E643:E681" ca="1" si="41">D643/12</f>
         <v>3.1249999999999997E-3</v>
       </c>
       <c r="F643">
@@ -41209,7 +41277,7 @@
         <v>182.09</v>
       </c>
       <c r="G644">
-        <f t="shared" ref="G644:G669" ca="1" si="43">C644/C643-1</f>
+        <f t="shared" ref="G644:G681" ca="1" si="43">C644/C643-1</f>
         <v>1.6968158395787025E-3</v>
       </c>
       <c r="H644">
@@ -41550,7 +41618,7 @@
       </c>
       <c r="J652">
         <f ca="1"/>
-        <v>74.362930000000006</v>
+        <v>75.993449999999996</v>
       </c>
     </row>
     <row r="653" spans="1:10" x14ac:dyDescent="0.25">
@@ -41591,7 +41659,7 @@
       </c>
       <c r="J653">
         <f ca="1"/>
-        <v>74.475790000000003</v>
+        <v>76.108800000000002</v>
       </c>
     </row>
     <row r="654" spans="1:10" x14ac:dyDescent="0.25">
@@ -41632,7 +41700,7 @@
       </c>
       <c r="J654">
         <f ca="1"/>
-        <v>74.752840000000006</v>
+        <v>76.391919999999999</v>
       </c>
     </row>
     <row r="655" spans="1:10" x14ac:dyDescent="0.25">
@@ -41673,7 +41741,7 @@
       </c>
       <c r="J655">
         <f ca="1"/>
-        <v>75.128079999999997</v>
+        <v>76.305400000000006</v>
       </c>
     </row>
     <row r="656" spans="1:10" x14ac:dyDescent="0.25">
@@ -41714,7 +41782,7 @@
       </c>
       <c r="J656">
         <f ca="1"/>
-        <v>75.535849999999996</v>
+        <v>76.719560000000001</v>
       </c>
     </row>
     <row r="657" spans="1:10" x14ac:dyDescent="0.25">
@@ -41755,7 +41823,7 @@
       </c>
       <c r="J657">
         <f ca="1"/>
-        <v>75.968969999999999</v>
+        <v>77.159469999999999</v>
       </c>
     </row>
     <row r="658" spans="1:10" x14ac:dyDescent="0.25">
@@ -41796,7 +41864,7 @@
       </c>
       <c r="J658">
         <f ca="1"/>
-        <v>76.341049999999996</v>
+        <v>77.537379999999999</v>
       </c>
     </row>
     <row r="659" spans="1:10" x14ac:dyDescent="0.25">
@@ -41837,7 +41905,7 @@
       </c>
       <c r="J659">
         <f ca="1"/>
-        <v>76.74924</v>
+        <v>77.95196</v>
       </c>
     </row>
     <row r="660" spans="1:10" x14ac:dyDescent="0.25">
@@ -41878,7 +41946,7 @@
       </c>
       <c r="J660">
         <f ca="1"/>
-        <v>77.287090000000006</v>
+        <v>78.498239999999996</v>
       </c>
     </row>
     <row r="661" spans="1:10" x14ac:dyDescent="0.25">
@@ -41919,7 +41987,7 @@
       </c>
       <c r="J661">
         <f ca="1"/>
-        <v>77.75573</v>
+        <v>78.974220000000003</v>
       </c>
     </row>
     <row r="662" spans="1:10" x14ac:dyDescent="0.25">
@@ -41960,7 +42028,7 @@
       </c>
       <c r="J662">
         <f ca="1"/>
-        <v>77.701859999999996</v>
+        <v>78.919510000000002</v>
       </c>
     </row>
     <row r="663" spans="1:10" x14ac:dyDescent="0.25">
@@ -42001,7 +42069,7 @@
       </c>
       <c r="J663">
         <f ca="1"/>
-        <v>77.808080000000004</v>
+        <v>79.0274</v>
       </c>
     </row>
     <row r="664" spans="1:10" x14ac:dyDescent="0.25">
@@ -42042,7 +42110,7 @@
       </c>
       <c r="J664">
         <f ca="1"/>
-        <v>78.082449999999994</v>
+        <v>79.306070000000005</v>
       </c>
     </row>
     <row r="665" spans="1:10" x14ac:dyDescent="0.25">
@@ -42083,7 +42151,7 @@
       </c>
       <c r="J665">
         <f ca="1"/>
-        <v>78.250529999999998</v>
+        <v>79.476780000000005</v>
       </c>
     </row>
     <row r="666" spans="1:10" x14ac:dyDescent="0.25">
@@ -42124,7 +42192,7 @@
       </c>
       <c r="J666">
         <f ca="1"/>
-        <v>78.497079999999997</v>
+        <v>79.727199999999996</v>
       </c>
     </row>
     <row r="667" spans="1:10" x14ac:dyDescent="0.25">
@@ -42165,7 +42233,7 @@
       </c>
       <c r="J667">
         <f ca="1"/>
-        <v>78.638620000000003</v>
+        <v>79.870949999999993</v>
       </c>
     </row>
     <row r="668" spans="1:10" x14ac:dyDescent="0.25">
@@ -42206,7 +42274,7 @@
       </c>
       <c r="J668">
         <f ca="1"/>
-        <v>78.902439999999999</v>
+        <v>80.138900000000007</v>
       </c>
     </row>
     <row r="669" spans="1:10" x14ac:dyDescent="0.25">
@@ -42238,7 +42306,7 @@
         <v>3.4826442022666271E-3</v>
       </c>
       <c r="H669">
-        <f t="shared" ca="1" si="42"/>
+        <f ca="1">E669-G669</f>
         <v>6.7355797733372694E-5</v>
       </c>
       <c r="I669">
@@ -42247,13 +42315,17 @@
       </c>
       <c r="J669">
         <f ca="1"/>
-        <v>79.057699999999997</v>
+        <v>80.296599999999998</v>
       </c>
     </row>
     <row r="670" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A670" t="str">
         <v>2025-09-30</v>
       </c>
+      <c r="B670">
+        <f t="shared" ca="1" si="40"/>
+        <v>234.55784283489336</v>
+      </c>
       <c r="C670">
         <f ca="1"/>
         <v>324.245</v>
@@ -42262,23 +42334,39 @@
         <f ca="1"/>
         <v>4.1200000000000001E-2</v>
       </c>
+      <c r="E670">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.4333333333333334E-3</v>
+      </c>
       <c r="F670">
         <f ca="1"/>
         <v>235.25</v>
       </c>
+      <c r="G670">
+        <f t="shared" ca="1" si="43"/>
+        <v>2.9509018191040681E-3</v>
+      </c>
+      <c r="H670">
+        <f t="shared" ref="H670:H680" ca="1" si="44">E670-G670</f>
+        <v>4.8243151422926525E-4</v>
+      </c>
       <c r="I670">
         <f ca="1"/>
         <v>1.6299999999999999E-2</v>
       </c>
       <c r="J670">
         <f ca="1"/>
-        <v>79.237440000000007</v>
+        <v>80.479150000000004</v>
       </c>
     </row>
     <row r="671" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A671" t="str">
         <v>2025-10-31</v>
       </c>
+      <c r="B671" t="e">
+        <f t="shared" ca="1" si="40"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="C671" t="str">
         <f ca="1"/>
         <v>ERR: NO DATA</v>
@@ -42287,9 +42375,21 @@
         <f ca="1"/>
         <v>4.0599999999999997E-2</v>
       </c>
+      <c r="E671">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.3833333333333332E-3</v>
+      </c>
       <c r="F671">
         <f ca="1"/>
-        <v>241.20332999999999</v>
+        <v>237.04467</v>
+      </c>
+      <c r="G671" t="e">
+        <f t="shared" ca="1" si="43"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H671" t="e">
+        <f t="shared" ca="1" si="44"/>
+        <v>#VALUE!</v>
       </c>
       <c r="I671">
         <f ca="1"/>
@@ -42297,13 +42397,17 @@
       </c>
       <c r="J671">
         <f ca="1"/>
-        <v>79.486620000000002</v>
+        <v>80.732240000000004</v>
       </c>
     </row>
     <row r="672" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A672" t="str">
         <v>2025-11-30</v>
       </c>
+      <c r="B672">
+        <f t="shared" ca="1" si="40"/>
+        <v>237.53735686629977</v>
+      </c>
       <c r="C672">
         <f ca="1"/>
         <v>325.06299999999999</v>
@@ -42312,9 +42416,21 @@
         <f ca="1"/>
         <v>4.0899999999999999E-2</v>
       </c>
+      <c r="E672">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.4083333333333331E-3</v>
+      </c>
       <c r="F672">
         <f ca="1"/>
-        <v>247.15666999999999</v>
+        <v>238.83932999999999</v>
+      </c>
+      <c r="G672" t="e">
+        <f t="shared" ca="1" si="43"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H672" t="e">
+        <f t="shared" ca="1" si="44"/>
+        <v>#VALUE!</v>
       </c>
       <c r="I672">
         <f ca="1"/>
@@ -42322,13 +42438,17 @@
       </c>
       <c r="J672">
         <f ca="1"/>
-        <v>80.104669999999999</v>
+        <v>81.359979999999993</v>
       </c>
     </row>
     <row r="673" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A673" t="str">
         <v>2025-12-31</v>
       </c>
+      <c r="B673">
+        <f t="shared" ca="1" si="40"/>
+        <v>238.61168568019602</v>
+      </c>
       <c r="C673">
         <f ca="1"/>
         <v>326.03100000000001</v>
@@ -42337,9 +42457,21 @@
         <f ca="1"/>
         <v>4.1399999999999999E-2</v>
       </c>
+      <c r="E673">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.4499999999999999E-3</v>
+      </c>
       <c r="F673">
         <f ca="1"/>
-        <v>253.11</v>
+        <v>240.63399999999999</v>
+      </c>
+      <c r="G673">
+        <f t="shared" ca="1" si="43"/>
+        <v>2.9778842870460398E-3</v>
+      </c>
+      <c r="H673">
+        <f t="shared" ca="1" si="44"/>
+        <v>4.7211571295396014E-4</v>
       </c>
       <c r="I673">
         <f ca="1"/>
@@ -42347,13 +42479,17 @@
       </c>
       <c r="J673">
         <f ca="1"/>
-        <v>80.472300000000004</v>
+        <v>81.733369999999994</v>
       </c>
     </row>
     <row r="674" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A674" t="str">
         <v>2026-01-31</v>
       </c>
+      <c r="B674">
+        <f t="shared" ca="1" si="40"/>
+        <v>245.16343386153193</v>
+      </c>
       <c r="C674">
         <f ca="1"/>
         <v>326.58800000000002</v>
@@ -42362,23 +42498,39 @@
         <f ca="1"/>
         <v>4.2099999999999999E-2</v>
       </c>
+      <c r="E674">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.5083333333333334E-3</v>
+      </c>
       <c r="F674">
         <f ca="1"/>
-        <v>261.30667</v>
+        <v>247.66367</v>
+      </c>
+      <c r="G674">
+        <f t="shared" ca="1" si="43"/>
+        <v>1.70842649932057E-3</v>
+      </c>
+      <c r="H674">
+        <f t="shared" ca="1" si="44"/>
+        <v>1.7999068340127634E-3</v>
       </c>
       <c r="I674">
         <f ca="1"/>
-        <v>1.54E-2</v>
+        <v>1.5299999999999999E-2</v>
       </c>
       <c r="J674">
         <f ca="1"/>
-        <v>80.266639999999995</v>
+        <v>81.720860000000002</v>
       </c>
     </row>
     <row r="675" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A675" t="str">
         <v>2026-02-28</v>
       </c>
+      <c r="B675">
+        <f t="shared" ca="1" si="40"/>
+        <v>251.45074619504675</v>
+      </c>
       <c r="C675">
         <f ca="1"/>
         <v>327.45999999999998</v>
@@ -42387,23 +42539,39 @@
         <f ca="1"/>
         <v>4.1300000000000003E-2</v>
       </c>
+      <c r="E675">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.4416666666666671E-3</v>
+      </c>
       <c r="F675">
         <f ca="1"/>
-        <v>269.50333000000001</v>
+        <v>254.69333</v>
+      </c>
+      <c r="G675">
+        <f t="shared" ca="1" si="43"/>
+        <v>2.6700307420970404E-3</v>
+      </c>
+      <c r="H675">
+        <f t="shared" ca="1" si="44"/>
+        <v>7.716359245696267E-4</v>
       </c>
       <c r="I675">
         <f ca="1"/>
-        <v>1.7000000000000001E-2</v>
+        <v>1.6899999999999998E-2</v>
       </c>
       <c r="J675">
         <f ca="1"/>
-        <v>79.980410000000006</v>
+        <v>81.624690000000001</v>
       </c>
     </row>
     <row r="676" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A676" t="str">
         <v>2026-03-31</v>
       </c>
+      <c r="B676">
+        <f t="shared" ca="1" si="40"/>
+        <v>256.17464007108839</v>
+      </c>
       <c r="C676">
         <f ca="1"/>
         <v>330.29300000000001</v>
@@ -42412,30 +42580,174 @@
         <f ca="1"/>
         <v>4.2500000000000003E-2</v>
       </c>
+      <c r="E676">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.5416666666666669E-3</v>
+      </c>
       <c r="F676">
         <f ca="1"/>
-        <v>277.7</v>
+        <v>261.72300000000001</v>
+      </c>
+      <c r="G676">
+        <f t="shared" ca="1" si="43"/>
+        <v>8.6514383436144815E-3</v>
+      </c>
+      <c r="H676">
+        <f t="shared" ca="1" si="44"/>
+        <v>-5.1097716769478146E-3</v>
       </c>
       <c r="I676">
         <f ca="1"/>
-        <v>1.67E-2</v>
+        <v>1.77E-2</v>
       </c>
       <c r="J676">
         <f ca="1"/>
-        <v>79.883359999999996</v>
+        <v>81.061530000000005</v>
       </c>
     </row>
     <row r="677" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A677" t="str">
         <v>2026-04-30</v>
       </c>
+      <c r="C677">
+        <f ca="1"/>
+        <v>332.40699999999998</v>
+      </c>
       <c r="D677">
         <f ca="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.3200000000000002E-2</v>
+      </c>
+      <c r="E677">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.6000000000000003E-3</v>
+      </c>
+      <c r="G677">
+        <f t="shared" ca="1" si="43"/>
+        <v>6.4003778463364025E-3</v>
+      </c>
+      <c r="H677">
+        <f t="shared" ca="1" si="44"/>
+        <v>-2.8003778463364022E-3</v>
       </c>
       <c r="I677">
         <f ca="1"/>
-        <v>1.6400000000000001E-2</v>
+        <v>1.66E-2</v>
+      </c>
+      <c r="J677">
+        <f ca="1"/>
+        <v>80.599710000000002</v>
+      </c>
+    </row>
+    <row r="678" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A678" t="str">
+        <v>2026-05-31</v>
+      </c>
+      <c r="C678">
+        <f ca="1"/>
+        <v>333.97899999999998</v>
+      </c>
+      <c r="D678">
+        <f ca="1"/>
+        <v>4.48E-2</v>
+      </c>
+      <c r="E678">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.7333333333333333E-3</v>
+      </c>
+      <c r="G678">
+        <f t="shared" ca="1" si="43"/>
+        <v>4.7291422864139676E-3</v>
+      </c>
+      <c r="H678">
+        <f t="shared" ca="1" si="44"/>
+        <v>-9.9580895308063432E-4</v>
+      </c>
+      <c r="I678">
+        <f ca="1"/>
+        <v>1.3899999999999999E-2</v>
+      </c>
+      <c r="J678">
+        <f ca="1"/>
+        <v>80.313969999999998</v>
+      </c>
+    </row>
+    <row r="679" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A679" t="str">
+        <v>2026-06-30</v>
+      </c>
+      <c r="C679">
+        <f ca="1"/>
+        <v>332.56799999999998</v>
+      </c>
+      <c r="D679">
+        <f ca="1"/>
+        <v>4.4699999999999997E-2</v>
+      </c>
+      <c r="E679">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.7249999999999996E-3</v>
+      </c>
+      <c r="G679">
+        <f t="shared" ca="1" si="43"/>
+        <v>-4.2248165303806484E-3</v>
+      </c>
+      <c r="H679">
+        <f t="shared" ca="1" si="44"/>
+        <v>7.9498165303806476E-3</v>
+      </c>
+      <c r="I679">
+        <f ca="1"/>
+        <v>1.3100000000000001E-2</v>
+      </c>
+      <c r="J679">
+        <f ca="1"/>
+        <v>80.816400000000002</v>
+      </c>
+    </row>
+    <row r="680" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A680" t="str">
+        <v>2026-07-31</v>
+      </c>
+      <c r="C680">
+        <f ca="1"/>
+        <v>332.81299999999999</v>
+      </c>
+      <c r="D680">
+        <f ca="1"/>
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="E680">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.8333333333333331E-3</v>
+      </c>
+      <c r="G680">
+        <f t="shared" ca="1" si="43"/>
+        <v>7.3669144355448246E-4</v>
+      </c>
+      <c r="H680">
+        <f t="shared" ca="1" si="44"/>
+        <v>3.0966418897788507E-3</v>
+      </c>
+      <c r="I680">
+        <f ca="1"/>
+        <v>1.18E-2</v>
+      </c>
+    </row>
+    <row r="681" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A681" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="D681">
+        <f ca="1"/>
+        <v>4.7500000000000001E-2</v>
+      </c>
+      <c r="E681">
+        <f t="shared" ca="1" si="41"/>
+        <v>3.9583333333333337E-3</v>
+      </c>
+      <c r="I681">
+        <f ca="1"/>
+        <v>9.7000000000000003E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>